<commit_message>
Version 0.2 Skin Processing
</commit_message>
<xml_diff>
--- a/Lab 2/bird_clock/素材与宣传清单.xlsx
+++ b/Lab 2/bird_clock/素材与宣传清单.xlsx
@@ -9,22 +9,23 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="故事线" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="素材表" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="宣传镜头" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能清单" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="进度" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="画布规格" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="素材表" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="宣传镜头" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能清单" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="进度" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'说明'!$1:$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'故事线'!$A$1:$I$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'故事线'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'素材表'!$A$1:$K$95</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'素材表'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'宣传镜头'!$A$1:$N$44</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'宣传镜头'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'功能清单'!$A$2:$G$20</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'功能清单'!$2:$2</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'进度'!$1:$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'素材表'!$A$1:$K$95</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'素材表'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'宣传镜头'!$A$1:$N$44</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'宣传镜头'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'功能清单'!$A$2:$G$20</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'功能清单'!$2:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'进度'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,6 +84,11 @@
       <name val="Arial"/>
       <color rgb="00008000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Menlo"/>
+      <color rgb="000000FF"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="9">
@@ -198,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -279,6 +285,19 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2299,6 +2318,391 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00BF8F00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="24" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>画布规格 · 照这个尺寸画就能直接进游戏</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>屏幕 240 x 135。全部 PNG，带透明通道，不要抗锯齿（引擎用 NEAREST 缩放，糊边会被放大）。放进 bird_clock/assets/&lt;皮肤名&gt;/ 就自动生效，缺文件就退回灰模。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>每类素材的画布</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>素材类型</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>画布尺寸</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>示例文件名</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>画的时候要注意什么</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>障碍（矩形类）</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>20 x 72</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>sprout.png / vine.png</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>宽度只会被缩到 14-20，高度 0-135 随机。顶端 18 像素是「不拉伸区」，树冠、藤蔓尖这些细节放这 18 像素里；其余部分会被拉伸，画成可重复的纹理</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>障碍（三角类）</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="inlineStr">
+        <is>
+          <t>20 x 72</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>hill.png / hill_down.png</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>整张等比缩放，不做三段切。画成三角剪影，四角留透明</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>连绵横条</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>16 x 18</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>caterpillar.png</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>横向无缝重复。左右两边要能接上，否则会看到接缝</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>拾取物</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="inlineStr">
+        <is>
+          <t>7 x 7</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>butterfly.png</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>很小，只能做剪影和两三个颜色。想画大一点就先跟我说，要改 ItemConfig.size</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>小鸟</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>8 x 8</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>bird.png</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>碰撞盒就是这 8x8，贴图别超出，否则看着撞到了其实没撞</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>天空</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>240 x 135</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>sky.png</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>整屏铺满，不滚动。也可以不放这张，只在 skin.json 里写一个背景色</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>远景层</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>120 x 135</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>far.png</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>横向无缝重复 + 视差滚动（默认 0.35 倍速）。左右边缘必须能接上</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>为什么障碍要留「不拉伸区」</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>障碍高度是随机的（28-72 像素连续变化），一张固定图直接拉伸会把树冠拉变形。所以引擎做三段切：贴着自由端的 18 像素原样保留，剩下的才拉伸。落地生长的障碍（新芽树），自由端在上；顶上垂下的（藤蔓），自由端在下。画的时候按它在游戏里的样子画就行，不用倒过来画。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>skin.json 怎么写</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="B20" s="34" t="inlineStr">
+        <is>
+          <t>{</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="13" customHeight="1">
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "background": "#BFE6F2",</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="13" customHeight="1">
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "sky": "sky.png",</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="13" customHeight="1">
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "far": "far.png",</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="13" customHeight="1">
+      <c r="B24" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "far_parallax": 0.35,</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="13" customHeight="1">
+      <c r="B25" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "obstacles": {</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="13" customHeight="1">
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "rect_bottom": {"file": "sprout.png", "cap": 18, "cap_at": "top"},</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "rect_top":    {"file": "vine.png",   "cap": 18, "cap_at": "bottom"},</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="13" customHeight="1">
+      <c r="B28" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "tri_bottom":  {"file": "hill.png"},</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="B29" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "tri_top":     {"file": "hill_down.png"},</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="13" customHeight="1">
+      <c r="B30" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "ground":      {"file": "caterpillar.png"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="13" customHeight="1">
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  },</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="13" customHeight="1">
+      <c r="B32" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "pickup": {"coin": "butterfly.png"},</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="13" customHeight="1">
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  "bird": "bird.png"</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="13" customHeight="1">
+      <c r="B34" s="34" t="inlineStr">
+        <is>
+          <t>}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>五个 obstacles 槽位可以少写：没写的槽位自动退回灰模方块，游戏照常跑。所以可以一次只画一个，边画边看。新做一个季节就复制整个文件夹改内容，再把 config.py 里 SkinConfig.name 改成新文件夹名。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>生成一套空白模板</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="34" t="inlineStr">
+        <is>
+          <t>python3 make_templates.py 夏天</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>会在 assets/ 下按上面所有尺寸生成占位图和 skin.json，直接覆盖着画即可。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="B36:H37"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B16:H17"/>
+    <mergeCell ref="B3:H3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00548235"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -6139,7 +6543,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -7986,14 +8390,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8114,12 +8518,12 @@
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>碰撞按类型共用，切换只换贴图与调色</t>
+          <t>已完成（基础版）：skin.json 换整套贴图；按时间自动选季节还没做，见 G06</t>
         </is>
       </c>
     </row>
@@ -8151,12 +8555,12 @@
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>现在只有单色背景</t>
+          <t>已完成：天空层 + 远景视差层，都不参与碰撞</t>
         </is>
       </c>
     </row>
@@ -8299,12 +8703,12 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>240x135 很小，预缩放一次即可</t>
+          <t>已完成：PNG 预缩放并缓存，缓存上限 512 条，实测 0.4ms/帧</t>
         </is>
       </c>
     </row>
@@ -8463,6 +8867,25 @@
       <c r="F20" s="12" t="n"/>
       <c r="G20" s="12" t="n"/>
     </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <autoFilter ref="A2:G20"/>
   <mergeCells count="1">
@@ -8486,7 +8909,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C65911"/>

</xml_diff>